<commit_message>
Se agrega tiempo entre llegadas y algunos cambios de la visualizacion de datos
</commit_message>
<xml_diff>
--- a/Heurística 3/Resultados/Resultados Calibración 2.0/ResultadosComparativos.xlsx
+++ b/Heurística 3/Resultados/Resultados Calibración 2.0/ResultadosComparativos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antonioalexxander/Desktop/Memoria/Experimentos Ideas/Heurística 3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antonioalexxander/Desktop/Memoria/Experimentos Ideas/Heurística 3/Resultados/Resultados Calibración 2.0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94C44510-D15A-E749-A327-A76D06C145E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50D7FF8-F665-7042-A5BE-F7F16F1136A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="2" xr2:uid="{990C28CB-0CE9-6947-BEC0-6C54E378B431}"/>
   </bookViews>
@@ -23,7 +23,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Datos!$A$1:$X$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -47,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="88">
   <si>
     <t>Mes</t>
   </si>
@@ -308,6 +307,9 @@
   </si>
   <si>
     <t>Global</t>
+  </si>
+  <si>
+    <t>Operación Manual</t>
   </si>
 </sst>
 </file>
@@ -6105,13 +6107,13 @@
       </c>
       <c r="O4" s="1"/>
       <c r="P4" s="24" t="s">
-        <v>10</v>
+        <v>87</v>
       </c>
       <c r="Q4" s="24"/>
       <c r="R4" s="24"/>
       <c r="S4" s="24"/>
       <c r="T4" s="24" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="U4" s="24"/>
       <c r="V4" s="24"/>

</xml_diff>